<commit_message>
revised stakeholder (citizens) analysis
</commit_message>
<xml_diff>
--- a/MCDA_Ratings_Werkspoor.xlsx
+++ b/MCDA_Ratings_Werkspoor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Amit/Documents/GitHub/Structural-group-5/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D85B58D-B248-134F-ACDE-2F7918FE05F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C438EE-28AC-114A-8E4F-E0AEE8DB3926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2320" yWindow="500" windowWidth="26480" windowHeight="16060" xr2:uid="{26C83A51-C2F9-474F-A238-2673A092AE5B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="78">
   <si>
     <t>MCDA Gold Coast Design Alternatives</t>
   </si>
@@ -249,6 +249,27 @@
   </si>
   <si>
     <t>existing transit infrastructure will need to be renovated to accommodate increased demand, can potentially affect visual appeal of area</t>
+  </si>
+  <si>
+    <t>Werkspoor bridge</t>
+  </si>
+  <si>
+    <t>Criteria Weight</t>
+  </si>
+  <si>
+    <t>Werkppoor bridge</t>
+  </si>
+  <si>
+    <t>alternate rail lines running during revovation of demka bridge</t>
+  </si>
+  <si>
+    <t>will increase line capacity after demka is renovated</t>
+  </si>
+  <si>
+    <t>lots of steel required, though not as much as the truss bridge</t>
+  </si>
+  <si>
+    <t>very pretty bridge</t>
   </si>
 </sst>
 </file>
@@ -1109,7 +1130,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2E21EC2-64DE-445B-8154-60469756B239}">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
@@ -1121,14 +1142,15 @@
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="20.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5" customWidth="1"/>
-    <col min="13" max="13" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1640625" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" customWidth="1"/>
+    <col min="16" max="16" width="15" customWidth="1"/>
+    <col min="17" max="17" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1136,7 +1158,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1165,22 +1187,25 @@
         <v>2</v>
       </c>
       <c r="L2" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" t="s">
         <v>36</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>37</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>40</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>41</v>
       </c>
-      <c r="P2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1212,19 +1237,22 @@
         <v>100</v>
       </c>
       <c r="M3">
+        <v>100</v>
+      </c>
+      <c r="N3">
         <v>80</v>
       </c>
-      <c r="N3">
-        <v>100</v>
-      </c>
       <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
         <v>40</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1253,22 +1281,25 @@
         <v>17</v>
       </c>
       <c r="L4">
+        <v>90</v>
+      </c>
+      <c r="M4">
         <v>60</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>80</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>90</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>70</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -1297,22 +1328,25 @@
         <v>39</v>
       </c>
       <c r="L5">
+        <v>50</v>
+      </c>
+      <c r="M5">
         <v>40</v>
       </c>
-      <c r="M5">
-        <v>100</v>
-      </c>
       <c r="N5">
+        <v>100</v>
+      </c>
+      <c r="O5">
         <v>50</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>30</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1344,19 +1378,22 @@
         <v>80</v>
       </c>
       <c r="M6">
+        <v>80</v>
+      </c>
+      <c r="N6">
         <v>10</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>80</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>30</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -1385,22 +1422,25 @@
         <v>22</v>
       </c>
       <c r="L7">
+        <v>60</v>
+      </c>
+      <c r="M7">
         <v>50</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>90</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>50</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>60</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1429,22 +1469,25 @@
         <v>42</v>
       </c>
       <c r="L8">
+        <v>70</v>
+      </c>
+      <c r="M8">
         <v>80</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>95</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>50</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>60</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1467,7 +1510,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -1490,7 +1533,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1513,7 +1556,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1536,7 +1579,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1559,7 +1602,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1581,11 +1624,11 @@
       <c r="G14" t="s">
         <v>29</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1608,7 +1651,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -1634,7 +1677,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1663,22 +1706,25 @@
         <v>2</v>
       </c>
       <c r="L17" t="s">
+        <v>73</v>
+      </c>
+      <c r="M17" t="s">
         <v>36</v>
       </c>
-      <c r="M17" t="s">
+      <c r="N17" t="s">
         <v>37</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>40</v>
       </c>
-      <c r="O17" t="s">
+      <c r="P17" t="s">
         <v>41</v>
       </c>
-      <c r="P17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1707,22 +1753,25 @@
         <v>35</v>
       </c>
       <c r="L18" t="s">
+        <v>74</v>
+      </c>
+      <c r="M18" t="s">
         <v>46</v>
       </c>
-      <c r="M18" t="s">
+      <c r="N18" t="s">
         <v>44</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>45</v>
       </c>
-      <c r="O18" t="s">
+      <c r="P18" t="s">
         <v>52</v>
       </c>
-      <c r="P18">
+      <c r="Q18">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J19" t="s">
         <v>38</v>
       </c>
@@ -1730,22 +1779,25 @@
         <v>17</v>
       </c>
       <c r="L19" t="s">
+        <v>51</v>
+      </c>
+      <c r="M19" t="s">
         <v>47</v>
       </c>
-      <c r="M19" t="s">
+      <c r="N19" t="s">
         <v>49</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>51</v>
       </c>
-      <c r="O19" t="s">
+      <c r="P19" t="s">
         <v>53</v>
       </c>
-      <c r="P19">
+      <c r="Q19">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J20" t="s">
         <v>38</v>
       </c>
@@ -1753,22 +1805,25 @@
         <v>39</v>
       </c>
       <c r="L20" t="s">
+        <v>62</v>
+      </c>
+      <c r="M20" t="s">
         <v>60</v>
       </c>
-      <c r="M20" t="s">
+      <c r="N20" t="s">
         <v>61</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>62</v>
       </c>
-      <c r="O20" t="s">
+      <c r="P20" t="s">
         <v>63</v>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J21" t="s">
         <v>38</v>
       </c>
@@ -1776,22 +1831,25 @@
         <v>54</v>
       </c>
       <c r="L21" t="s">
+        <v>75</v>
+      </c>
+      <c r="M21" t="s">
         <v>55</v>
       </c>
-      <c r="M21" t="s">
+      <c r="N21" t="s">
         <v>56</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>58</v>
       </c>
-      <c r="O21" t="s">
+      <c r="P21" t="s">
         <v>59</v>
       </c>
-      <c r="P21">
+      <c r="Q21">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J22" t="s">
         <v>38</v>
       </c>
@@ -1799,22 +1857,25 @@
         <v>22</v>
       </c>
       <c r="L22" t="s">
+        <v>76</v>
+      </c>
+      <c r="M22" t="s">
         <v>64</v>
       </c>
-      <c r="M22" t="s">
+      <c r="N22" t="s">
         <v>65</v>
       </c>
-      <c r="N22" t="s">
+      <c r="O22" t="s">
         <v>66</v>
       </c>
-      <c r="O22" t="s">
+      <c r="P22" t="s">
         <v>67</v>
       </c>
-      <c r="P22">
+      <c r="Q22">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="J23" t="s">
         <v>38</v>
       </c>
@@ -1822,18 +1883,21 @@
         <v>42</v>
       </c>
       <c r="L23" t="s">
+        <v>77</v>
+      </c>
+      <c r="M23" t="s">
         <v>68</v>
       </c>
-      <c r="M23" t="s">
+      <c r="N23" t="s">
         <v>69</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>57</v>
       </c>
-      <c r="O23" t="s">
+      <c r="P23" t="s">
         <v>70</v>
       </c>
-      <c r="P23">
+      <c r="Q23">
         <v>10</v>
       </c>
     </row>

</xml_diff>